<commit_message>
Update Integrated Disclosure 2026-10-13
</commit_message>
<xml_diff>
--- a/Integrated_Disclosure_Report.xlsx
+++ b/Integrated_Disclosure_Report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,6 +488,58 @@
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t>계약(수주)일자</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AI데이터센터연료전지용울트라캐패시터(UC)공급계약</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>미해당</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>68880240000</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>68880240000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>44.85</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>iConnexionAsiaPteLtd.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2027-04-16</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2028-03-17</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Integrated Disclosure 2026-10-20
</commit_message>
<xml_diff>
--- a/Integrated_Disclosure_Report.xlsx
+++ b/Integrated_Disclosure_Report.xlsx
@@ -554,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -636,90 +636,90 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>13300418504</v>
+        <v>123010501824</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>13300418504</v>
+        <v>123010501824</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>16.17</v>
+        <v>149.6</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>SANMINACORPORATION</t>
+          <t>ACBELPOLYTECHINC</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2027-01-28</t>
+          <t>2028-02-01</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
+          <t>주권매매거래정지              (단일판매공급계약)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>데이터센터용슈퍼커패시터공급계약</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>미해당</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>38361874110</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>38361874110</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>46.65</v>
+        <v>0</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ACBELPOLYTECHINC</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2027-03-15</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -740,19 +740,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>13112996702</v>
+        <v>13300418504</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>13112996702</v>
+        <v>13300418504</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>15.95</v>
+        <v>16.17</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -761,17 +761,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2027-01-28</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>데이터센터용슈퍼커패시터시스템공급계약</t>
+          <t>데이터센터용슈퍼커패시터공급계약</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -792,50 +792,50 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>41215393800</v>
+        <v>38361874110</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>41215393800</v>
+        <v>38361874110</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>50.12</v>
+        <v>46.65</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BloomEnergyCorporation</t>
+          <t>ACBELPOLYTECHINC</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2027-04-10</t>
+          <t>2027-03-15</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
+          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
+          <t>데이터센터용슈퍼커패시터공급계약</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -844,38 +844,38 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10104945135</v>
+        <v>13112996702</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>10104945135</v>
+        <v>13112996702</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>16.96</v>
+        <v>15.95</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ACBELPOLYTECHINC</t>
+          <t>SANMINACORPORATION</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -887,45 +887,149 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>데이터센터용슈퍼커패시터시스템공급계약</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>미해당</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>41215393800</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>41215393800</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>50.12</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>BloomEnergyCorporation</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2027-04-10</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>미해당</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D8" t="n">
+        <v>10104945135</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>10104945135</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ACBELPOLYTECHINC</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>미해당</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
         <v>6758155342</v>
       </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
         <v>6758155342</v>
       </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
         <v>11.34</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>ACBELPOLYTECHINC</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>2025-06-13</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>2025-09-30</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>2025-06-13</t>
         </is>

</xml_diff>

<commit_message>
Update Integrated Disclosure 2026-10-22
</commit_message>
<xml_diff>
--- a/Integrated_Disclosure_Report.xlsx
+++ b/Integrated_Disclosure_Report.xlsx
@@ -554,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -636,38 +636,38 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>123010501824</v>
+        <v>119474738573</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>123010501824</v>
+        <v>119474738573</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>149.6</v>
+        <v>145.3</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ACBELPOLYTECHINC</t>
+          <t>SANMINACORPORATION</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2028-02-01</t>
+          <t>2027-12-23</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -740,90 +740,90 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>13300418504</v>
+        <v>123010501824</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>13300418504</v>
+        <v>123010501824</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>16.17</v>
+        <v>149.6</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>SANMINACORPORATION</t>
+          <t>ACBELPOLYTECHINC</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2027-01-28</t>
+          <t>2028-02-01</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
+          <t>주권매매거래정지              (단일판매공급계약)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>데이터센터용슈퍼커패시터공급계약</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>미해당</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>38361874110</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>38361874110</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>46.65</v>
+        <v>0</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>ACBELPOLYTECHINC</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2027-03-15</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -844,19 +844,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>13112996702</v>
+        <v>13300418504</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>13112996702</v>
+        <v>13300418504</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>15.95</v>
+        <v>16.17</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -865,17 +865,17 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2027-01-28</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>데이터센터용슈퍼커패시터시스템공급계약</t>
+          <t>데이터센터용슈퍼커패시터공급계약</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -896,50 +896,50 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>41215393800</v>
+        <v>38361874110</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>41215393800</v>
+        <v>38361874110</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>50.12</v>
+        <v>46.65</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BloomEnergyCorporation</t>
+          <t>ACBELPOLYTECHINC</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2027-04-10</t>
+          <t>2027-03-15</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
+          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
+          <t>데이터센터용슈퍼커패시터공급계약</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -948,38 +948,38 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>10104945135</v>
+        <v>13112996702</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>10104945135</v>
+        <v>13112996702</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>16.96</v>
+        <v>15.95</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>ACBELPOLYTECHINC</t>
+          <t>SANMINACORPORATION</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -991,45 +991,149 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>데이터센터용슈퍼커패시터시스템공급계약</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>미해당</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>41215393800</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>41215393800</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>50.12</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>BloomEnergyCorporation</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2027-04-10</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[기재정정]단일판매ㆍ공급계약체결              </t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>미해당</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D10" t="n">
+        <v>10104945135</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10104945135</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>ACBELPOLYTECHINC</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">단일판매ㆍ공급계약체결              </t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>데이터센터비상전원용슈퍼커퍼시터(에너지저장장치)공급계약</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>미해당</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
         <v>6758155342</v>
       </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="n">
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
         <v>6758155342</v>
       </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
         <v>11.34</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>ACBELPOLYTECHINC</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>2025-06-13</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>2025-09-30</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>2025-06-13</t>
         </is>

</xml_diff>